<commit_message>
feat: district detail panel, building/wonder placement adjacency, DoNotDisplayWhenPlacement
- Add RUIVO_DISTRICT_DETAIL_PANEL (lua+xml) sliding left panel for district placement
- Support building/wonder placement adjacency via Ruivo_Building_District_Mapping table
- Add DoNotDisplayWhenPlacement parameter to suppress WORKER adjacencies in placement mode
- Add hasDistrict parameter to Ruivo_ExtraAdjacentYieldBonusString for placement vs built logic
- Add pcall protection for nil-plot StatsModule fallback
- Add MAB_TryApplyOverride in AdjacencyBonusSupport.lua via Events.LoadScreenClose
- Fix tutorial .md: DistrictModifiers 0->1 in ModifierOwner example (zh+en)
</commit_message>
<xml_diff>
--- a/!参考性文件(reference_folder)/refer_table-参考表/Ruivo_ModifierOwner_CollectionType.xlsx
+++ b/!参考性文件(reference_folder)/refer_table-参考表/Ruivo_ModifierOwner_CollectionType.xlsx
@@ -128,8 +128,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -145,7 +153,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -153,12 +161,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,16 +483,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>